<commit_message>
CR-030/031/032/033 : produit réel, organisé — plus de « démo »
- CR-030 (fait) : le concept démo disparaît de l'interface. « Essai gratuit »,
  « Essayer Coreon », « École d'exemple », « Journée simulée » ; textes serveur
  honnêtes (« aucun serveur connecté ») ; mobile aligné ; i18n arabe suit les
  nouvelles clés. 18/18 parcours e2e verts.
- CR-033 (fait) : Catalogue produit — Coreon-EDU_Product-Catalog.xlsx généré du
  code (nav/features/locales) par build-product-catalog.py : 35 modules avec web
  et mobile sur la même ligne, 16 services du cœur, rôles, 4 pays, intégrations.
- CR-031 (plan) : docs/operations/environments.md — dev → int → prod à la
  version finale, jamais de saut ; les 4 pays sont une couche de config, pas
  des branches.
- CR-034 (ouvert) : Porte d'intégration système enregistrée au classeur.
- Nettoyage : branche develop locale supprimée (stale, 66 en retard).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
+++ b/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
@@ -32139,7 +32139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T144"/>
+  <dimension ref="A1:T149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34802,7 +34802,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P30" s="16" t="inlineStr"/>
@@ -34811,7 +34811,7 @@
       <c r="S30" s="16" t="n"/>
       <c r="T30" s="16" t="inlineStr">
         <is>
-          <t>SPÉCIFIÉ 2026-07-23 : docs/quality/hr-accounting-module-spec.md §3 (recherche NetSuite/ERPNext/Focus/GCC). Séquencement §5. À construire un sous-module à la fois. Gap actuel : salaire mono-montant, pas de bulletin, pas de WPS/EOSB, pas d'organigramme.</t>
+          <t>Volet 1 livré 2026-07-25 (85fb30d) : salaire multi-composants, bulletin de paie, maker-checker.</t>
         </is>
       </c>
     </row>
@@ -37382,6 +37382,266 @@
       <c r="R144" s="16" t="n"/>
       <c r="S144" s="16" t="n"/>
       <c r="T144" s="16" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>CR-030</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Othman</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Produit réel</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Retirer le concept « démo » du produit</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>C'est un produit réel maintenant, pas une démonstration. Toute mention démo disparaît de l'interface (web + mobile).</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Tout le produit</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>Livré 2026-07-25 : CTA « Essai gratuit », « École d'exemple », « Journée simulée » ; i18n AR alignée ; 18/18 e2e verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>CR-031</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Othman</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Environnements</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>3 environnements GitHub : dev / int / prod</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>prod = ce que les clients reçoivent ; int = modifications client ; dev = développement. À créer à la préparation de la version finale.</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Dépôt / CI</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>TRIAGED</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>Plan écrit : docs/operations/environments.md. Déclenché par « version finale ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>CR-032</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Othman</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Versions pays</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>4 versions produit : Bahreïn, Tunisie, Qatar, Libye</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Le cadre permanent du produit. La couche pays existe (locales.js, CR-023/024) ; compléter curriculum/fériés/conformité par pays.</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Couche pays</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>BH/QA/TN/LY présents dans locales.js ; manques Tier-1 par pays dans gap-analysis.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>CR-033</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Othman</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Documentation produit</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Catalogue produit Excel : tous les éléments décrits</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Modules, services, rôles, comptes, pays, intégrations — web et mobile sur la même ligne.</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>docs/quality</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Livré 2026-07-25 : Coreon-EDU_Product-Catalog.xlsx + générateur build-product-catalog.py (régénérable du code).</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>CR-034</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Othman</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Intégrations</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Porte d'intégration système (import des données client)</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>La porte par laquelle un client apporte SES données : import OneRoster/CSV guidé (correspondance de colonnes, validation, rapport), puis API REST + webhooks.</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Intégrations</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>Demandé 2026-07-25. Après : l'hébergement backend. Export OneRoster + import JSON serveur existent déjà.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:T2"/>

</xml_diff>

<commit_message>
CR-031 → DONE dans le registre (environnements en place)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
+++ b/docs/quality/Coreon-EDU_QA-Test-Workbook.xlsx
@@ -37478,12 +37478,12 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>TRIAGED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="T146" t="inlineStr">
         <is>
-          <t>Plan écrit : docs/operations/environments.md. Déclenché par « version finale ».</t>
+          <t>Plan écrit : docs/operations/environments.md. Déclenché par « version finale ». · EN PLACE 2026-07-25 (version finale déclarée, 1er client BH) : branches dev/int + main=prod ; dev.edu + int.edu (Cloudflare Pages) ; envs.yml (dev rapide, int chaîne complète) ; environnements GitHub + protection main (checks requis) ; branche par défaut = dev ; secrets Cloudflare posés.</t>
         </is>
       </c>
     </row>

</xml_diff>